<commit_message>
Seattle map template: Watch cells are real embedded hyperlinks, visible immediately
Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0161jaxJZTksz7q1T7aevp9F
</commit_message>
<xml_diff>
--- a/lr-seattle-tv-map-rows.xlsx
+++ b/lr-seattle-tv-map-rows.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,6 +30,12 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001155CC"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -61,9 +67,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -468,7 +475,7 @@
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="44" customWidth="1" min="10" max="10"/>
     <col width="9" customWidth="1" min="11" max="11"/>
     <col width="8" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
@@ -572,9 +579,10 @@
           <t>Get LNR_15</t>
         </is>
       </c>
-      <c r="G2" s="2">
-        <f>HYPERLINK("https://wdvcseovujheftpzcoer.supabase.co/storage/v1/object/public/creative/SEALR2615003T.mp4","▶ Watch")</f>
-        <v/>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>▶ Watch</t>
+        </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
@@ -629,9 +637,10 @@
           <t>If Your Wreck_15</t>
         </is>
       </c>
-      <c r="G3" s="2">
-        <f>HYPERLINK("https://wdvcseovujheftpzcoer.supabase.co/storage/v1/object/public/creative/SEALR2615004T.mp4","▶ Watch")</f>
-        <v/>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>▶ Watch</t>
+        </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
@@ -690,9 +699,10 @@
           <t>Ins Stop_15</t>
         </is>
       </c>
-      <c r="G4" s="2">
-        <f>HYPERLINK("https://wdvcseovujheftpzcoer.supabase.co/storage/v1/object/public/creative/SEALR2615005T.mp4","▶ Watch")</f>
-        <v/>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>▶ Watch</t>
+        </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
@@ -702,7 +712,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Cites 2014 insurance study (ethics caveat)</t>
+          <t>Cites 2014 insurance study - ethics business-risk caveat</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -751,9 +761,10 @@
           <t>Wreck Check_15</t>
         </is>
       </c>
-      <c r="G5" s="2">
-        <f>HYPERLINK("https://wdvcseovujheftpzcoer.supabase.co/storage/v1/object/public/creative/SEALR2615006T.mp4","▶ Watch")</f>
-        <v/>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>▶ Watch</t>
+        </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
@@ -812,9 +823,10 @@
           <t>Overnight_15</t>
         </is>
       </c>
-      <c r="G6" s="2">
-        <f>HYPERLINK("https://wdvcseovujheftpzcoer.supabase.co/storage/v1/object/public/creative/SEALR2615010T.mp4","▶ Watch")</f>
-        <v/>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>▶ Watch</t>
+        </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
@@ -869,9 +881,10 @@
           <t>Weekend_15</t>
         </is>
       </c>
-      <c r="G7" s="2">
-        <f>HYPERLINK("https://wdvcseovujheftpzcoer.supabase.co/storage/v1/object/public/creative/SEALR2615011T.mp4","▶ Watch")</f>
-        <v/>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>▶ Watch</t>
+        </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
@@ -913,6 +926,14 @@
       <formula>$C2=TRUE</formula>
     </cfRule>
   </conditionalFormatting>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>